<commit_message>
Enhance v1.9: Rotate secondary off-day across months for 4-day/week staff with 1 fixed off-day (Miyazawa)
</commit_message>
<xml_diff>
--- a/26年10-12月シフト.xlsx
+++ b/26年10-12月シフト.xlsx
@@ -863,14 +863,14 @@
           <t>公</t>
         </is>
       </c>
-      <c r="T3" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="U3" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="T3" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="U3" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V3" s="8">
@@ -892,9 +892,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA3" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA3" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB3" s="8" t="inlineStr">
@@ -907,9 +907,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD3" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD3" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE3" s="8" t="inlineStr">
@@ -954,19 +954,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
@@ -979,9 +979,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
@@ -1057,9 +1057,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC4" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD4" s="8" t="inlineStr">
@@ -1067,9 +1067,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AE4" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AF4" s="11" t="inlineStr">
@@ -1119,9 +1119,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
@@ -1149,18 +1149,18 @@
           <t>公</t>
         </is>
       </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="O5" s="8">
         <f>COUNTIF(E5:N5, "○")</f>
         <v/>
       </c>
-      <c r="Q5" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="Q5" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="R5" s="8" t="inlineStr">
@@ -1168,9 +1168,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S5" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="T5" s="8" t="inlineStr">
@@ -1475,9 +1475,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="T7" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="T7" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U7" s="8" t="inlineStr">
@@ -1504,9 +1504,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA7" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA7" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB7" s="8" t="inlineStr">
@@ -1519,14 +1519,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD7" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="AE7" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AD7" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="AE7" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AF7" s="8" t="inlineStr">
@@ -1630,14 +1630,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T8" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="U8" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T8" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="U8" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V8" s="8">
@@ -1679,9 +1679,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE8" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AE8" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AF8" s="8" t="inlineStr">
@@ -1721,19 +1721,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
@@ -1746,9 +1746,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L9" s="8" t="inlineStr">
@@ -1780,14 +1780,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S9" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T9" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S9" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T9" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U9" s="8" t="inlineStr">
@@ -1824,9 +1824,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC9" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AC9" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AD9" s="8" t="inlineStr">
@@ -1945,9 +1945,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U10" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U10" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V10" s="8">
@@ -1969,9 +1969,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA10" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA10" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB10" s="8" t="inlineStr">
@@ -1984,9 +1984,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD10" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD10" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE10" s="8" t="inlineStr">
@@ -2035,19 +2035,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H11" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
@@ -2060,9 +2060,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K11" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L11" s="15" t="inlineStr">
@@ -2099,9 +2099,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T11" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U11" s="15" t="inlineStr">
@@ -2138,9 +2138,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC11" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC11" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD11" s="15" t="inlineStr">
@@ -2148,9 +2148,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AE11" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AF11" s="11" t="inlineStr">
@@ -2190,9 +2190,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -2230,9 +2230,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="N12" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="O12" s="8">
@@ -2699,14 +2699,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T15" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="U15" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T15" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="U15" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V15" s="8">
@@ -2728,9 +2728,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA15" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA15" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB15" s="8" t="inlineStr">
@@ -2748,9 +2748,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE15" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AE15" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AF15" s="8" t="inlineStr">
@@ -2794,19 +2794,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F16" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G16" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
@@ -2819,9 +2819,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K16" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L16" s="15" t="inlineStr">
@@ -2897,14 +2897,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC16" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="AD16" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC16" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="AD16" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE16" s="15" t="inlineStr">
@@ -3018,9 +3018,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U17" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U17" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V17" s="8">
@@ -3042,9 +3042,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA17" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA17" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB17" s="8" t="inlineStr">
@@ -3057,9 +3057,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD17" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD17" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE17" s="8" t="inlineStr">
@@ -3108,19 +3108,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H18" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
@@ -3133,9 +3133,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K18" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L18" s="15" t="inlineStr">
@@ -3172,9 +3172,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T18" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U18" s="15" t="inlineStr">
@@ -3211,9 +3211,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC18" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC18" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD18" s="15" t="inlineStr">
@@ -3221,9 +3221,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AE18" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AF18" s="11" t="inlineStr">
@@ -3654,9 +3654,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA21" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA21" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB21" s="8" t="inlineStr">
@@ -3669,9 +3669,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD21" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AD21" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE21" s="8" t="inlineStr">
@@ -3780,14 +3780,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T22" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="U22" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T22" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="U22" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V22" s="8">
@@ -3829,9 +3829,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE22" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AE22" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AF22" s="8" t="inlineStr">
@@ -3871,19 +3871,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
@@ -3896,9 +3896,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K23" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L23" s="8" t="inlineStr">
@@ -3974,9 +3974,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC23" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AC23" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AD23" s="8" t="inlineStr">
@@ -4095,9 +4095,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U24" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U24" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V24" s="8">
@@ -4119,9 +4119,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA24" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA24" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB24" s="8" t="inlineStr">
@@ -4134,9 +4134,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD24" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD24" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE24" s="8" t="inlineStr">
@@ -4185,19 +4185,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H25" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I25" s="15" t="inlineStr">
@@ -4210,9 +4210,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K25" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L25" s="15" t="inlineStr">
@@ -4249,9 +4249,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T25" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T25" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U25" s="15" t="inlineStr">
@@ -4288,9 +4288,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC25" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC25" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD25" s="15" t="inlineStr">
@@ -4298,9 +4298,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE25" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AE25" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AF25" s="11" t="inlineStr">
@@ -4345,9 +4345,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -4360,9 +4360,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="J26" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="K26" s="8" t="inlineStr">
@@ -4399,9 +4399,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S26" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S26" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="T26" s="8" t="inlineStr">
@@ -4697,9 +4697,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S28" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S28" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="T28" s="8" t="inlineStr">
@@ -4707,9 +4707,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U28" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="U28" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V28" s="8">
@@ -4731,9 +4731,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA28" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA28" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB28" s="8" t="inlineStr">
@@ -4741,14 +4741,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC28" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="AD28" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC28" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="AD28" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE28" s="8" t="inlineStr">
@@ -4861,9 +4861,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T29" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="T29" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U29" s="15" t="inlineStr">
@@ -4890,9 +4890,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA29" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA29" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB29" s="15" t="inlineStr">
@@ -4910,9 +4910,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE29" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AE29" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AF29" s="15" t="inlineStr">
@@ -4952,19 +4952,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H30" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr">
@@ -4977,9 +4977,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K30" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K30" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L30" s="8" t="inlineStr">
@@ -5001,9 +5001,9 @@
         <f>COUNTIF(E30:N30, "○")</f>
         <v/>
       </c>
-      <c r="Q30" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="Q30" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="R30" s="8" t="inlineStr">
@@ -5055,14 +5055,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC30" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="AD30" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC30" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="AD30" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE30" s="8" t="inlineStr">
@@ -5200,9 +5200,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA31" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA31" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB31" s="8" t="inlineStr">
@@ -5215,9 +5215,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD31" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD31" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE31" s="8" t="inlineStr">
@@ -5262,19 +5262,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G32" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H32" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
@@ -5287,9 +5287,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K32" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L32" s="11" t="inlineStr">
@@ -5321,14 +5321,14 @@
           <t>公</t>
         </is>
       </c>
-      <c r="S32" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T32" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S32" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T32" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U32" s="8" t="inlineStr">
@@ -5365,9 +5365,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC32" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC32" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD32" s="8" t="inlineStr">
@@ -5375,9 +5375,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AE32" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AE32" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AF32" s="11" t="inlineStr">
@@ -5437,14 +5437,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="J33" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="K33" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="K33" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
@@ -5476,14 +5476,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S33" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="T33" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S33" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="T33" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U33" s="11" t="inlineStr">
@@ -5863,112 +5863,112 @@
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
+          <t>水</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>水</t>
+        </is>
+      </c>
+      <c r="H37" s="17" t="inlineStr">
+        <is>
           <t>金</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="I37" s="17" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="J37" s="17" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="H37" s="17" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="I37" s="17" t="inlineStr">
+      <c r="L37" s="17" t="inlineStr">
+        <is>
+          <t>火・月</t>
+        </is>
+      </c>
+      <c r="M37" s="17" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="Q37" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="R37" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="S37" s="17" t="inlineStr">
         <is>
           <t>木</t>
         </is>
       </c>
-      <c r="J37" s="17" t="inlineStr">
+      <c r="T37" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="U37" s="17" t="inlineStr">
+        <is>
+          <t>土・木</t>
+        </is>
+      </c>
+      <c r="X37" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y37" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z37" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA37" s="17" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="AB37" s="17" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="AC37" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="AD37" s="17" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="K37" s="17" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="L37" s="17" t="inlineStr">
+      <c r="AE37" s="17" t="inlineStr">
         <is>
           <t>火</t>
-        </is>
-      </c>
-      <c r="M37" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="N37" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="Q37" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="R37" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
-        </is>
-      </c>
-      <c r="S37" s="17" t="inlineStr">
-        <is>
-          <t>木</t>
-        </is>
-      </c>
-      <c r="T37" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
-        </is>
-      </c>
-      <c r="U37" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="X37" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y37" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z37" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA37" s="17" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="AB37" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="AC37" s="17" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="AD37" s="17" t="inlineStr">
-        <is>
-          <t>木</t>
-        </is>
-      </c>
-      <c r="AE37" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
         </is>
       </c>
       <c r="AF37" s="17" t="inlineStr">
@@ -6368,9 +6368,9 @@
       </c>
       <c r="C4" s="9" t="inlineStr"/>
       <c r="D4" s="10" t="inlineStr"/>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -6403,9 +6403,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -6442,9 +6442,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="U4" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V4" s="8">
@@ -6466,9 +6466,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA4" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB4" s="8" t="inlineStr">
@@ -6476,9 +6476,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC4" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD4" s="8" t="inlineStr">
@@ -6679,19 +6679,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H6" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
@@ -6704,9 +6704,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K6" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L6" s="15" t="inlineStr">
@@ -6738,9 +6738,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S6" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S6" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="T6" s="15" t="inlineStr">
@@ -6829,14 +6829,14 @@
       </c>
       <c r="C7" s="9" t="inlineStr"/>
       <c r="D7" s="10" t="inlineStr"/>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -6844,9 +6844,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
@@ -6864,9 +6864,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L7" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -6898,14 +6898,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T7" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="U7" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T7" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="U7" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V7" s="8">
@@ -6998,9 +6998,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -7018,9 +7018,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L8" s="15" t="inlineStr">
@@ -7086,9 +7086,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA8" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA8" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB8" s="15" t="inlineStr">
@@ -7096,9 +7096,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC8" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AC8" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AD8" s="11" t="inlineStr">
@@ -7476,9 +7476,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -7510,14 +7510,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="U11" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="T11" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V11" s="8">
@@ -7596,9 +7596,9 @@
       </c>
       <c r="C12" s="9" t="inlineStr"/>
       <c r="D12" s="10" t="inlineStr"/>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -7660,14 +7660,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S12" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="T12" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S12" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="T12" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U12" s="8" t="inlineStr">
@@ -7694,9 +7694,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA12" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA12" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB12" s="8" t="inlineStr">
@@ -7704,9 +7704,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC12" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC12" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD12" s="8" t="inlineStr">
@@ -7756,19 +7756,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -7781,9 +7781,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L13" s="8" t="inlineStr">
@@ -7815,14 +7815,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S13" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T13" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T13" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U13" s="8" t="inlineStr">
@@ -7906,14 +7906,14 @@
       </c>
       <c r="C14" s="9" t="inlineStr"/>
       <c r="D14" s="10" t="inlineStr"/>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -7921,9 +7921,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -7941,9 +7941,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -7975,14 +7975,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T14" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="U14" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T14" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="U14" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V14" s="8">
@@ -8075,9 +8075,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -8095,9 +8095,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L15" s="15" t="inlineStr">
@@ -8163,9 +8163,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA15" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA15" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB15" s="15" t="inlineStr">
@@ -8173,9 +8173,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC15" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AC15" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AD15" s="11" t="inlineStr">
@@ -8284,14 +8284,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S16" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="T16" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="T16" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U16" s="11" t="inlineStr">
@@ -8553,9 +8553,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -8587,14 +8587,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="U18" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="T18" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="U18" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V18" s="8">
@@ -8673,9 +8673,9 @@
       </c>
       <c r="C19" s="9" t="inlineStr"/>
       <c r="D19" s="10" t="inlineStr"/>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -8771,9 +8771,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA19" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA19" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB19" s="8" t="inlineStr">
@@ -8781,9 +8781,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC19" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC19" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD19" s="8" t="inlineStr">
@@ -8837,19 +8837,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I20" s="15" t="inlineStr">
@@ -8862,9 +8862,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K20" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L20" s="15" t="inlineStr">
@@ -8896,14 +8896,14 @@
           <t>特有</t>
         </is>
       </c>
-      <c r="S20" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T20" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S20" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T20" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U20" s="15" t="inlineStr">
@@ -8987,14 +8987,14 @@
       </c>
       <c r="C21" s="9" t="inlineStr"/>
       <c r="D21" s="10" t="inlineStr"/>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -9002,9 +9002,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
@@ -9022,9 +9022,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="L21" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M21" s="8" t="inlineStr">
@@ -9056,14 +9056,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T21" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="U21" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T21" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="U21" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V21" s="8">
@@ -9156,9 +9156,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H22" s="15" t="inlineStr">
@@ -9176,9 +9176,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K22" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="L22" s="15" t="inlineStr">
@@ -9244,9 +9244,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA22" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA22" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB22" s="15" t="inlineStr">
@@ -9254,9 +9254,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC22" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AC22" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AD22" s="11" t="inlineStr">
@@ -9746,9 +9746,9 @@
       </c>
       <c r="C26" s="9" t="inlineStr"/>
       <c r="D26" s="10" t="inlineStr"/>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -9815,9 +9815,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="T26" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="T26" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U26" s="8" t="inlineStr">
@@ -9844,9 +9844,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA26" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA26" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB26" s="8" t="inlineStr">
@@ -9854,9 +9854,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC26" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC26" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD26" s="8" t="inlineStr">
@@ -9906,19 +9906,19 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="H27" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="I27" s="8" t="inlineStr">
@@ -9931,9 +9931,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K27" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K27" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L27" s="8" t="inlineStr">
@@ -10056,14 +10056,14 @@
       </c>
       <c r="C28" s="9" t="inlineStr"/>
       <c r="D28" s="10" t="inlineStr"/>
-      <c r="E28" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -10071,9 +10071,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
@@ -10091,9 +10091,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L28" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="L28" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -10221,9 +10221,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
@@ -10241,14 +10241,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K29" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="L29" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="L29" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M29" s="8" t="inlineStr">
@@ -10285,9 +10285,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U29" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="U29" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V29" s="8">
@@ -10309,9 +10309,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AA29" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA29" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB29" s="8" t="inlineStr">
@@ -10319,9 +10319,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC29" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AC29" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AD29" s="11" t="inlineStr">
@@ -10420,9 +10420,9 @@
         <f>COUNTIF(E30:N30, "○")</f>
         <v/>
       </c>
-      <c r="Q30" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="Q30" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="R30" s="8" t="inlineStr">
@@ -10430,9 +10430,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S30" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S30" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="T30" s="8" t="inlineStr">
@@ -10718,9 +10718,9 @@
         <f>COUNTIF(E32:N32, "○")</f>
         <v/>
       </c>
-      <c r="Q32" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="Q32" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="R32" s="8" t="inlineStr">
@@ -10738,9 +10738,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="U32" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U32" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V32" s="8">
@@ -11110,107 +11110,107 @@
       </c>
       <c r="E36" s="17" t="inlineStr">
         <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
           <t>木</t>
         </is>
       </c>
-      <c r="F36" s="17" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="H36" s="17" t="inlineStr">
         <is>
           <t>水</t>
         </is>
       </c>
-      <c r="G36" s="17" t="inlineStr">
+      <c r="I36" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="J36" s="17" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="K36" s="17" t="inlineStr">
         <is>
           <t>水</t>
         </is>
       </c>
-      <c r="H36" s="17" t="inlineStr">
+      <c r="L36" s="17" t="inlineStr">
+        <is>
+          <t>火・木</t>
+        </is>
+      </c>
+      <c r="M36" s="17" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="N36" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="Q36" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="R36" s="17" t="inlineStr">
         <is>
           <t>木</t>
         </is>
       </c>
-      <c r="I36" s="17" t="inlineStr">
+      <c r="S36" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="T36" s="17" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="U36" s="17" t="inlineStr">
+        <is>
+          <t>土・月</t>
+        </is>
+      </c>
+      <c r="X36" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y36" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z36" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA36" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="AB36" s="17" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="AC36" s="17" t="inlineStr">
         <is>
           <t>火</t>
-        </is>
-      </c>
-      <c r="J36" s="17" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="K36" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
-        </is>
-      </c>
-      <c r="L36" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="M36" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="N36" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
-        </is>
-      </c>
-      <c r="Q36" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="R36" s="17" t="inlineStr">
-        <is>
-          <t>木</t>
-        </is>
-      </c>
-      <c r="S36" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
-        </is>
-      </c>
-      <c r="T36" s="17" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="U36" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="X36" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y36" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z36" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA36" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="AB36" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="AC36" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
         </is>
       </c>
       <c r="AD36" s="17" t="inlineStr">
@@ -11482,14 +11482,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
@@ -11507,9 +11507,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L3" s="11" t="inlineStr">
@@ -11541,14 +11541,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T3" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S3" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T3" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U3" s="8" t="inlineStr">
@@ -11575,9 +11575,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA3" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA3" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB3" s="8" t="inlineStr">
@@ -11590,9 +11590,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD3" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD3" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE3" s="8" t="inlineStr">
@@ -11666,14 +11666,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="L4" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="L4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M4" s="15" t="inlineStr">
@@ -11700,9 +11700,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="S4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S4" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="T4" s="15" t="inlineStr">
@@ -11734,9 +11734,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA4" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA4" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB4" s="15" t="inlineStr">
@@ -11759,9 +11759,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AF4" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AF4" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AG4" s="15" t="inlineStr">
@@ -11855,9 +11855,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S5" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S5" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="T5" s="8" t="inlineStr">
@@ -11899,14 +11899,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC5" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="AD5" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC5" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="AD5" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE5" s="8" t="inlineStr">
@@ -11955,14 +11955,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -12014,14 +12014,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S6" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="T6" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S6" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="T6" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U6" s="15" t="inlineStr">
@@ -12058,9 +12058,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC6" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC6" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD6" s="15" t="inlineStr">
@@ -12073,9 +12073,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AF6" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AF6" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AG6" s="15" t="inlineStr">
@@ -12438,9 +12438,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L9" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -12563,14 +12563,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -12588,9 +12588,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K10" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
@@ -12622,14 +12622,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S10" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T10" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S10" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T10" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U10" s="8" t="inlineStr">
@@ -12656,9 +12656,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA10" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA10" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB10" s="8" t="inlineStr">
@@ -12671,9 +12671,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD10" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD10" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE10" s="8" t="inlineStr">
@@ -12743,14 +12743,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="L11" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -12777,9 +12777,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="S11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S11" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="T11" s="8" t="inlineStr">
@@ -12787,9 +12787,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U11" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U11" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V11" s="8">
@@ -12811,9 +12811,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA11" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA11" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB11" s="8" t="inlineStr">
@@ -12836,9 +12836,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AF11" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AF11" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AG11" s="8" t="inlineStr">
@@ -12932,9 +12932,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S12" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S12" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="T12" s="8" t="inlineStr">
@@ -12942,9 +12942,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U12" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="U12" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V12" s="8">
@@ -12976,14 +12976,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC12" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="AD12" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC12" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="AD12" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE12" s="8" t="inlineStr">
@@ -13032,14 +13032,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -13091,14 +13091,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S13" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="T13" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S13" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="T13" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U13" s="15" t="inlineStr">
@@ -13135,9 +13135,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC13" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC13" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD13" s="15" t="inlineStr">
@@ -13150,9 +13150,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AF13" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AF13" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AG13" s="15" t="inlineStr">
@@ -13515,9 +13515,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L16" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -13644,14 +13644,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G17" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -13669,9 +13669,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K17" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
@@ -13703,14 +13703,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S17" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T17" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S17" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T17" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U17" s="15" t="inlineStr">
@@ -13737,9 +13737,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA17" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA17" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB17" s="15" t="inlineStr">
@@ -13752,9 +13752,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD17" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD17" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE17" s="15" t="inlineStr">
@@ -13824,14 +13824,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="L18" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -13858,9 +13858,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="S18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S18" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="T18" s="8" t="inlineStr">
@@ -13868,9 +13868,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U18" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U18" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V18" s="8">
@@ -13892,9 +13892,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA18" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA18" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB18" s="8" t="inlineStr">
@@ -13917,9 +13917,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AF18" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AF18" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AG18" s="8" t="inlineStr">
@@ -14013,9 +14013,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S19" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S19" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="T19" s="8" t="inlineStr">
@@ -14023,9 +14023,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U19" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="U19" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V19" s="8">
@@ -14057,14 +14057,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC19" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="AD19" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC19" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="AD19" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE19" s="8" t="inlineStr">
@@ -14113,14 +14113,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -14172,14 +14172,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S20" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="T20" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S20" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="T20" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U20" s="15" t="inlineStr">
@@ -14216,9 +14216,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC20" s="15" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC20" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD20" s="15" t="inlineStr">
@@ -14231,9 +14231,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AF20" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AF20" s="15" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AG20" s="15" t="inlineStr">
@@ -14596,9 +14596,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L23" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M23" s="8" t="inlineStr">
@@ -14721,14 +14721,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -14746,9 +14746,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="L24" s="11" t="inlineStr">
@@ -14780,14 +14780,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S24" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="T24" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S24" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="T24" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="U24" s="8" t="inlineStr">
@@ -14814,9 +14814,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA24" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AA24" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AB24" s="8" t="inlineStr">
@@ -14829,9 +14829,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AD24" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AD24" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AE24" s="8" t="inlineStr">
@@ -14901,14 +14901,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="M25" s="8" t="inlineStr">
@@ -14935,9 +14935,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="S25" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="S25" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="T25" s="8" t="inlineStr">
@@ -14945,9 +14945,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U25" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="U25" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="V25" s="8">
@@ -14969,9 +14969,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AA25" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AA25" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AB25" s="8" t="inlineStr">
@@ -14994,9 +14994,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AF25" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AF25" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AG25" s="8" t="inlineStr">
@@ -15090,9 +15090,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S26" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S26" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="T26" s="8" t="inlineStr">
@@ -15100,9 +15100,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="U26" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="U26" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="V26" s="8">
@@ -15134,14 +15134,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC26" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="AD26" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC26" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="AD26" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AE26" s="8" t="inlineStr">
@@ -15186,14 +15186,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
@@ -15245,14 +15245,14 @@
           <t>○</t>
         </is>
       </c>
-      <c r="S27" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
-        </is>
-      </c>
-      <c r="T27" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="S27" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="T27" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="U27" s="8" t="inlineStr">
@@ -15289,9 +15289,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="AC27" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="AC27" s="11" t="inlineStr">
+        <is>
+          <t>公</t>
         </is>
       </c>
       <c r="AD27" s="8" t="inlineStr">
@@ -15304,9 +15304,9 @@
           <t>公</t>
         </is>
       </c>
-      <c r="AF27" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="AF27" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="AG27" s="8" t="inlineStr">
@@ -15669,9 +15669,9 @@
           <t>○</t>
         </is>
       </c>
-      <c r="L30" s="11" t="inlineStr">
-        <is>
-          <t>公</t>
+      <c r="L30" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -16562,117 +16562,117 @@
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
           <t>火</t>
         </is>
       </c>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="H37" s="17" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="H37" s="17" t="inlineStr">
+      <c r="I37" s="17" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="J37" s="17" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="L37" s="17" t="inlineStr">
+        <is>
+          <t>火・水</t>
+        </is>
+      </c>
+      <c r="M37" s="17" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>水</t>
+        </is>
+      </c>
+      <c r="Q37" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="R37" s="17" t="inlineStr">
+        <is>
+          <t>水</t>
+        </is>
+      </c>
+      <c r="S37" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="T37" s="17" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="I37" s="17" t="inlineStr">
+      <c r="U37" s="17" t="inlineStr">
+        <is>
+          <t>土・水</t>
+        </is>
+      </c>
+      <c r="X37" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y37" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z37" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA37" s="17" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="AB37" s="17" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="AC37" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="AD37" s="17" t="inlineStr">
         <is>
           <t>木</t>
         </is>
       </c>
-      <c r="J37" s="17" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="K37" s="17" t="inlineStr">
+      <c r="AE37" s="17" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="AF37" s="17" t="inlineStr">
         <is>
           <t>水</t>
-        </is>
-      </c>
-      <c r="L37" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="M37" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="N37" s="17" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="Q37" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="R37" s="17" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="S37" s="17" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="T37" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="U37" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="X37" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y37" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z37" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA37" s="17" t="inlineStr">
-        <is>
-          <t>水</t>
-        </is>
-      </c>
-      <c r="AB37" s="17" t="inlineStr">
-        <is>
-          <t>土</t>
-        </is>
-      </c>
-      <c r="AC37" s="17" t="inlineStr">
-        <is>
-          <t>木</t>
-        </is>
-      </c>
-      <c r="AD37" s="17" t="inlineStr">
-        <is>
-          <t>火</t>
-        </is>
-      </c>
-      <c r="AE37" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
-        </is>
-      </c>
-      <c r="AF37" s="17" t="inlineStr">
-        <is>
-          <t>金</t>
         </is>
       </c>
       <c r="AG37" s="17" t="inlineStr">

</xml_diff>